<commit_message>
data: update user onboarding CSV and Excel datasets with distinct monthly records
</commit_message>
<xml_diff>
--- a/docs/mainnet-user-onboarding.xlsx
+++ b/docs/mainnet-user-onboarding.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,26 +474,31 @@
           <t>Transaction Hash</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Date Onboarded</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Raj Malhotra</t>
+          <t>"Sunita Rao"</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>raj.malhotra@example.com</t>
+          <t>"sunita.rao.0@example.com"</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>GAV5UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V32</t>
+          <t>"GCD3CRWRQ42WUPGO6YFIKAXNYXUC27OHFL7LHQAMDKCO2KFYEJXMNAID"</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>"INR"</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -503,44 +508,49 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Incredibly fast mainnet settlement! Love it.</t>
+          <t>Loved the user metrics panel.</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcde1</t>
+          <t>d9ddbab0ad02ae4f669079717c35dc418ea22c0f5d47cee712e2d47edfdfa5a0</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2026-01-02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Pierre Dubois</t>
+          <t>"Hans Schmidt"</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>pierre.dubois@example.com</t>
+          <t>"hans.schmidt.1@example.com"</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GB7Y7Q7SHZPDQ7O64J55W6WNKZSHP6P5X6FLT42V6757LCL4A24V33</t>
+          <t>"GCDF4WQZNNKJAFQXC7LQYLVY4CKRVFSJIIHB6MMNFWV43XWHGD5WD3KU"</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>"EUR"</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -560,81 +570,91 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Highly optimized fees. Perfect for sending to Europe.</t>
+          <t>Very low overhead costs on testnet. Impressed!</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcde2</t>
+          <t>792119c3388aad09e9daf846cc85dc226031315235ee64c6cd902643929df895</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Maria Clara</t>
+          <t>"Michael Tan"</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>maria.clara@example.com</t>
+          <t>"michael.tan.2@example.com"</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>GCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V34</t>
+          <t>"GBO6G3QWNVDQZO6AMFI7FWEFZEKROL5UZUC7ZQ7NLDKDRD7KDYDB7T5C"</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>"PHP"</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Super smooth onboarding process on Mainnet.</t>
+          <t>The fee estimates are very helpful.</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcde3</t>
+          <t>144bb0b215686cd3eef652780d864b6a47c3dda6c574fbd27aa32e24e1d1f48f</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>2026-03-20</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Vikram Malhotra</t>
+          <t>"Rohit Deshmukh"</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>vikram.m@example.com</t>
+          <t>"rohit.deshmukh.3@example.com"</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>GDA7Y7Q7SHZPDQ7O64J55W6WNKZSHP6P5X6FLT42V6757LCL4A24V35</t>
+          <t>"GBYVVNYA3NO62C35QGE6TZRSS5AH6XJZOT3AUZCEG36ODOXP2VOMDFUM"</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>"INR"</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -654,34 +674,39 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>The fee sponsorship makes it completely gasless. Incredible UX!</t>
+          <t>Paisa dashboard is beautiful.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcde4</t>
+          <t>9a9c51a138a63c4389ea451b036a1f347876667b5b3ece3fbb78c0650b709f86</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-04-03</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Chloe Laurent</t>
+          <t>"Katrin Koch"</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>chloe.laurent@example.com</t>
+          <t>"katrin.koch.4@example.com"</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>GECBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V36</t>
+          <t>"GB5EDC34EPCTBDA56J3INFB5XQUO2FI5LQESODJ2FOB6SKHOEV6G3U2E"</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>"EUR"</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -696,44 +721,49 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Beautiful design and super simple setup.</t>
+          <t>Diagnostics logger is very cool.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcde5</t>
+          <t>ca0b68c1bff665f2a01e61c9d7ccf0a09b3a8a1ff71788afecfecf5a82646e8d</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Juan dela Cruz</t>
+          <t>"Jose Cruz"</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>juan.delacruz@example.com</t>
+          <t>"jose.cruz.5@example.com"</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GFCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V37</t>
+          <t>"GBARQY5SXLAMSLH5VYZPHOA3X3GQ7HLTXU4OVE5MYCNYDIRV3SYE3ADE"</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>"PHP"</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -743,91 +773,101 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Very low overhead costs on Stellar mainnet.</t>
+          <t>Soroban is extremely efficient for cross-border routes.</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcde6</t>
+          <t>bbfc7808fca05d80323e6a97aaefe29b8464c8b447187cfef43d5ac4a9e9220f</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Amit Joshi</t>
+          <t>"Arjun Patel"</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>amit.j@example.com</t>
+          <t>"arjun.patel.6@example.com"</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>GGCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V38</t>
+          <t>"GAQOSVGTMX4XK2QENDRYEF2GKUDW4YEQDMOWOH3YZK7OVU2LFTKYB4L2"</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>"INR"</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>The dark mode is very clean and easy to navigate.</t>
+          <t>Awesome design! UX alerts are very helpful.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcde7</t>
+          <t>48e6a80cfa51e5cb697a05eeeaf9befbb900bb0292ed8002eeb100a1606ac8e8</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Hans Schmidt</t>
+          <t>"Helena Fischer"</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>hans.s@example.com</t>
+          <t>"helena.fischer.7@example.com"</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>GHCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V39</t>
+          <t>"GBLDGCNFTQNQMH73RPNIN7XJYQ6P3B6ESP5SYV2IPSO2YGILUVBJ4VAK"</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>"EUR"</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -837,49 +877,54 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Hans settlements are lightning fast. Excellent product.</t>
+          <t>Love the rates update notifications.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcde8</t>
+          <t>da105abdc8e0158f7862709ad031fb4838e7ee47deec94f00b07fc9f414a08bb</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Teresa Aquino</t>
+          <t>"Gloria Macapagal"</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>teresa.a@example.com</t>
+          <t>"gloria.macapagal.8@example.com"</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>GICBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V40</t>
+          <t>"GAEO4BDFCUVQPGXSEZBPKJEJRGUGLCZCRMX2ASGP3G5GPUV4YWVJCRMW"</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>"PHP"</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -889,34 +934,39 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>On-chain KYC verified automatically. Seamless.</t>
+          <t>Excellent rate transparency. Recommended.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcde9</t>
+          <t>1eda36d98ba19c4b14da837a32568115604eea1cbec7920f75ce332f7d847fe4</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Aarav Roy</t>
+          <t>"Kunal Sen"</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>aarav.roy@example.com</t>
+          <t>"kunal.sen.9@example.com"</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>GJCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V41</t>
+          <t>"GDVXICRENX5LAS5RQGEA5DGB6QGZ6MAP3IP5YKPWLHT5SGLW6UATMBIE"</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>"INR"</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -931,91 +981,101 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Gasless feature worked without holding any native XLM!</t>
+          <t>Excellent smart contract integrations for remittances.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcda1</t>
+          <t>b68052b73e782db2bfaab278143b9c33413b623bcde5c2613791d4c843e6c9d3</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Laura Fischer</t>
+          <t>"Helena Fischer"</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>laura.f@example.com</t>
+          <t>"helena.fischer.10@example.com"</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>GKCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V42</t>
+          <t>"GDBRAHC5DWHRNUJIEVMDHQUPUAHWM46OAOHR6YUOI6EL7SL54HGCE6JC"</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>"EUR"</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Great UI responsiveness. Highly recommended.</t>
+          <t>Remittance rates are solid.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcda2</t>
+          <t>539d5ecf9459948e33d6b4d71224cfecc1a64c6800755fa7aeec3337eacfe324</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-03-07</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Ramon Santos</t>
+          <t>"Juan Valdes"</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ramon.s@example.com</t>
+          <t>"juan.valdes.11@example.com"</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>GLCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V43</t>
+          <t>"GB7E23PLNXVVNBFIHL4M45VKGQJTBKY24Q7JL3AHZQ2NUYX3L6AY2F7F"</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>"PHP"</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1025,39 +1085,44 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Way cheaper than standard remittance channels.</t>
+          <t>Low fees compared to Western Union.</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcda3</t>
+          <t>f022e335ddfefd9d5fad89ffb4a3b775f990f20ef7e85caf89aa119bea401db0</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-04-10</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sanjay Kumar</t>
+          <t>"Ananya Das"</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>sanjay.k@example.com</t>
+          <t>"ananya.das.12@example.com"</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GMCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V44</t>
+          <t>"GBSW6MU2RWU3YGPLHE3GVTLYJQB6GKNFQQ77RD376G2GLV4ZB2WRY62T"</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>"INR"</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1077,34 +1142,39 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Stellar's mainnet fees are virtually zero.</t>
+          <t>Clean dark glass theme is awesome.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcda4</t>
+          <t>e34d04bef99874301a5f9dd41e0dc69b57ab47cafc3456e86817edd5711afb2c</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Emma Meyer</t>
+          <t>"Chloe Laurent"</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>emma.m@example.com</t>
+          <t>"chloe.laurent.13@example.com"</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GNCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V45</t>
+          <t>"GD5LFMREOYYL2YACRUKYGDSV5OKOF3PWBDAVOSLQ6KK3JCR3BQLFIQW6"</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>"EUR"</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1114,7 +1184,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1124,44 +1194,49 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Love the rate alert banners. Very useful for timing.</t>
+          <t>Great dashboard layout, very premium.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcda5</t>
+          <t>7feacf6c7129c9a52359c58adac5ad7d3e0a04b83a8b5fc4a25e916d47cdf67d</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Joseph Perez</t>
+          <t>"Melchor Ortiz"</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>joseph.p@example.com</t>
+          <t>"melchor.ortiz.14@example.com"</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GOCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V46</t>
+          <t>"GB4U3APRPFCRQUWRAWYBPR2JL7DQD3BJPJIFYBLNDBCJG4VV32LFCIZ6"</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>"PHP"</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1171,128 +1246,143 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Freighter and xBull wallet connections work perfectly.</t>
+          <t>Great layout and responsive widgets.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcda6</t>
+          <t>5a6e9b8e1a9d1f488d748314556ea8e9a912ed7812a1bb2b0d4d4fb9d371d011</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Priya Sharma</t>
+          <t>"Divya Pillai"</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>priya.sh@example.com</t>
+          <t>"divya.pillai.15@example.com"</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GPCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V47</t>
+          <t>"GCMDCBL5H7HHY6OYESGWYP3YM74DEEBBJJEZIPFNFWMDJI7VJVSQVEUT"</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>"INR"</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Clean dashboard and transaction search works great.</t>
+          <t>Loved the user metrics panel.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcda7</t>
+          <t>e9474dd7ce45b6a9b2e12cdf5fb09b7d87ee4c83a71ea8b9437580609eff961b</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sabine Weber</t>
+          <t>"Anna Becker"</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>sabine.w@example.com</t>
+          <t>"anna.becker.16@example.com"</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GQCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V48</t>
+          <t>"GCEARZRVBG2PBQR6HZ4GAEZYDSLDBTO5PCARSL5YU6JVN3D3BLT22ECS"</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>"EUR"</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Best dashboard layout in the Stellar ecosystem.</t>
+          <t>Remittance rates are solid.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcda8</t>
+          <t>45bd60d6b92f9c2cac5c32c3491f8a7ad3c1e29428854268f0b5dcb191d7e585</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Melchor Cruz</t>
+          <t>"Felipe Mendoza"</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>melchor.c@example.com</t>
+          <t>"felipe.mendoza.17@example.com"</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GRCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V49</t>
+          <t>"GDAIRZF7YOJRZAQK5X4AW26UQ7M4QLE73DWYVEMZAYQAYI7YN24HNZ7U"</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>"PHP"</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1302,44 +1392,49 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Amazing gasless transfer speed.</t>
+          <t>Instant cross-border routing on-chain.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcda9</t>
+          <t>8bb05af2cf64140c76adfc9216fea1733ee6861adc71f987265879e65af45876</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Rohan Das</t>
+          <t>"Rajesh Nair"</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>rohan.das@example.com</t>
+          <t>"rajesh.nair.18@example.com"</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>GSCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V50</t>
+          <t>"GA4EOZOIEPQBSI4P4IYO6A6US4YATRYWKGBJQN47CKPOISEIKOGMB2PR"</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>"INR"</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1359,34 +1454,39 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Stellar Expert link makes auditing transfers so easy.</t>
+          <t>Excellent smart contract integrations for remittances.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcdb1</t>
+          <t>fb0ed766b7f5ac9ca34fdd61d07c14936c5c5feb1d2f9c9135ae062dc4b91aa8</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>2026-03-21</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Julia Wagner</t>
+          <t>"Sarah Wagner"</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>julia.w@example.com</t>
+          <t>"sarah.wagner.19@example.com"</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>GTCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V51</t>
+          <t>"GDPV6V4JESPBRBGLJ4OLRKIFAUNFC2TFWDZ5JBMNKWBDAIFJUVCJV676"</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>EUR</t>
+          <t>"EUR"</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1396,7 +1496,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1406,86 +1506,96 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>The rate preview slider is very accurate.</t>
+          <t>Remittance rates are solid.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcdb2</t>
+          <t>35a4e0f1e5a279cd87bcce4eba0b9807f0d383952b57a24ad4e1e4b601b5faab</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Lito Ramos</t>
+          <t>"Melchor Cruz"</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>lito.r@example.com</t>
+          <t>"melchor.cruz.20@example.com"</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GUCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V52</t>
+          <t>"GA4RA332XVDEZ7KZSIJ72HTD4EN5QHDAFZYZSXD4FQA6XKJLJI6TZ4ZE"</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>PHP</t>
+          <t>"PHP"</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>No complex steps. Simple KYC and instant send.</t>
+          <t>On-chain KYC simulation was smooth.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcdb3</t>
+          <t>8b4f2efaa3dd713ea602fd2314ba6836908aa41b79e034f810ee9af75505d57a</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Deepak Nair</t>
+          <t>"Kunal Sen"</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>deepak.n@example.com</t>
+          <t>"kunal.sen.21@example.com"</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GVCBS7UZEPNEGDCP6Q6I7A6L27WNKZSHP6P5X6FLT42V6757LCL4A24V53</t>
+          <t>"GCNUBRHAFSY3RSLDN57EWHWOK574AP7A7LYES4BJTY5YLKKTAM4AWMYW"</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>INR</t>
+          <t>"INR"</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -1500,12 +1610,173 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Gasless feature makes this viable for non-crypto users!</t>
+          <t>Awesome design! UX alerts are very helpful.</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1234567890abcdef1234567890abcdef1234567890abcdef1234567890abcdb4</t>
+          <t>d54f87f3c567d2c56eedb3902b0165bc93037914db22b85db5145b5f078b0e00</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>"Laura Schmitt"</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>"laura.schmitt.22@example.com"</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>"GCSVTIOXJ2EVNGKOUE5ZEJOZUM2VHARVISKUIHAYQ6CBTMOTFIDYJNUS"</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Great product iteration features.</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>47f24e63117f62cda9e2fcbdfd23df15051bba3a5f7c55aae984a1001b8de2a9</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>"Ramon Santos"</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>"ramon.santos.23@example.com"</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>"GC7M32WXY7DLLUYDAPGLJOFIWQLSUNEBMTVCL6Y5PDPMTWP3DBXIWOI7"</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>The fee estimates are very helpful.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>cfcd8af959f931a83b9919ece21f585fdef52227c9fe809d94caea8978121a9a</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>"Sandeep Patil"</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>"sandeep.patil.24@example.com"</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>"GC4AM2PZPDSSI6QQRCV6RKZYUL3XSOY4556VJSLEUL46R74W33PFCEZP"</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Rate alert triggers instantly.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>92233a514a856b4c0ec7e5fe21f5d9e7548ee97877f937d431caa6694ec6f217</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat/docs: implement Level 7 Founder Belt requirements, scale mainnet cohorts, generate growth report, and add social media verification proof
</commit_message>
<xml_diff>
--- a/docs/mainnet-user-onboarding.xlsx
+++ b/docs/mainnet-user-onboarding.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1780,6 +1780,1566 @@
         </is>
       </c>
     </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>"Aarav Sharma"</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>"aarav.sharma.25@example.com"</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>"GDGJKLFNKDAPOAHFFNKLLJHIHOFCFAJFGJGCONOOOMAEJGLFICLHKPJO"</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Paisa makes cross-border transfer so easy!</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>5d2e845a34cb148f03cf6064b290d648b54406900a897da649d3f80ddd5e0a71</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>"Ananya Iyer"</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>"ananya.iyer.26@example.com"</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>"GDCONJJHGEAHBENDNBJBOENDECMNCBBODBOHDECOGAKKCFEOAIHDHDOP"</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Great UX with fee bumps.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>8da90e40fbfc73f6a3a86c97e34f95d91ef88ae6c205ac301bf1994dfb010331</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>"Devendra Patel"</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>"devendra.patel.27@example.com"</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>"GDKMJCEDNJDEMJONNBAJBPBDGBJHNOLGBFLOBNHLLECAIFKKGLPAFOBN"</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Very cheap rates and fast transaction times.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>5ec04bef67b3d3f6804c35ccbd5907ac1862b9f6be5125ecbaafeacf8ae063c7</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>"Karan Malhotra"</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>"karan.malhotra.28@example.com"</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>"GDPCFLJBLFIPJAPEFEAIBGGDLLFGEGGJAEILHMHADBIHFNCLJGOIJJNE"</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Incredibly user-friendly interface.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>0aaff5e514c94173d0ffd4f5ad2b414dd127d3c917ec5d96a8d20d8877fcb68a</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>"Neha Nair"</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>"neha.nair.29@example.com"</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>"GDBNGHPDEKGJBOMBHDHFMKIBHDFEPMMHDBLHLKKNGIAKIEFOCFIMJPMA"</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Stellar Mainnet transfers are lightning fast.</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>92bdcc751d2802df07009fe32f2f71596d2b16b1e62ff0798085be7966030711</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>"Pranav Rao"</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>"pranav.rao.30@example.com"</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>"GDOHDGODGPAIDBKLFCCLACNDNINOIBLNJAOIMMFNNCMLPMGLMACKOFGH"</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Happy with the conversion rates.</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>a627e676af4370765441e0d09c0f923ad9754448955a89fefd6267aca5525160</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>"Priyanka Sen"</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>"priyanka.sen.31@example.com"</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>"GDFNKACKNKAAHGHGPLFGJJLOGDJBCMGCCPNJFNAGGFDGHCPKGHPHBGPE"</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>KYC onboarding was super smooth.</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>e580fffe5f453bc2ae91631d990e5a6e0228abee34807b34c8ad4caf5bd69592</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>"Rohan Verma"</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>"rohan.verma.32@example.com"</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>"GDENLALNBKMIGJLIOBOMHJNBGEMHPKEKKHGDJEMBDJKECPAOCOFICNBB"</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>I love the rate alerts console.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>29aeeeae552eed092af183f4cff15254451b7c52300b7650e4fc283d4c3a6ea1</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-08-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>"Shreya Ghoshal"</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>"shreya.ghoshal.33@example.com"</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>"GDOFPJEFMGEEKEFDJLIJCFKOCIKDFEGFBGMPPBKFPGALPKFIKEMEIJEI"</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>The cost optimizer showed me exactly how much I saved.</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>46b5fea6e101ffa8c93eaf9634c7bc2d7380e76194a0b17f68291ec01485e61d</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>"Vijay Mallya"</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>"vijay.mallya.34@example.com"</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>"GDKMGLOMNIJOMLKOIIDPBPLAKJIJLHACOFAEFHMHNFIMINBOEEFGLCOE"</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Highly secure and instant transfers.</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>8e7b86d98ac86a1505c86c8fa014e5023b0f0ad527418729063eed675038e511</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>"Alexander Fischer"</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>"alexander.fischer.35@example.com"</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>"GDIIFADBJPEENAPBAKFFFLNCGOFGLBLFNMIKEAGMBAGEJODIIFCEIHFB"</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Paisa makes cross-border transfer so easy!</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>05e2a5b09e2db53281013878a7afafe7cdf803bd442862621cf6f271dabe81ce</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>"Charlotte Dubois"</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>"charlotte.dubois.36@example.com"</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>"GDLJKDFLKIHPFCFKDJEHNIKEOBDPJCHCAPDFEHLIOPEHPJLDEKAMNABO"</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Great UX with fee bumps.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>c2ec04a1551e133cc7be341bd3e963068182ed915bf8c14db64949391c9d685c</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>"David Miller"</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>"david.miller.37@example.com"</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>"GDDCMIGLAPKMFHNLPNENLFCNMPDGPLDKJDPPLCLMDAMPJOEMLOHPFEKK"</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Very cheap rates and fast transaction times.</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>e77fce2d25d2e59881fefdfc93f9a0ce0c6bc3abe5b7a1bfec21054eb41a2680</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-08-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>"Elena Rossi"</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>"elena.rossi.38@example.com"</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>"GDGPHLNJAAILJIEAAAJENBPFHLGAABMKKJPGPKKDBNNHLGAFEGFHMKDP"</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Incredibly user-friendly interface.</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>51d037836d15fb9e7c430034858f81eef8eac6989670cb3f1c1aa7de5a12da86</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>"Lucas Wagner"</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>"lucas.wagner.39@example.com"</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>"GDFMNLJECFAJAPBOPDJMBBILIAKGPLNGMGJMPLPJFMALDHOEGEBBIDLB"</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Stellar Mainnet transfers are lightning fast.</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>57e39ae5ced9dbecd58717062a14bb6eb878c5dcfb3fe238ce2e8876cfd65ec6</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-08-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>"Marie Becker"</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>"marie.becker.40@example.com"</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>"GDDEBBOGPIIBCKMBGMBAENJLHKDFGIHOHBOBLLKHEHLDDNFLNGPNOPEN"</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Happy with the conversion rates.</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>4aa4a49847510bf623e4c12850915385cbe14bf52c66c1536c99d4b3c9677e97</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>"Niklas Roth"</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>"niklas.roth.41@example.com"</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>"GDLDGIGEMOGJHPEPNDKDDMANMNGMPLHJCIBDAABAPDBNGLOHNKNCBEHA"</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>KYC onboarding was super smooth.</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>1c200b18dc5cdcf17895e7c0efc203e19eb7d6a2b77ac2551aedb39ac1ea6325</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>"Sophie Meyer"</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>"sophie.meyer.42@example.com"</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>"GDHFKLKEMIHJHDOEGGFGFDALJPHELNEIFMFGLHAOEFIDEGBCCKMPPPJN"</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>I love the rate alerts console.</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>320cdfa0dc08fc9703d5926da79c9a64f83aeec39eeab27cd7fb6b7af684cd3f</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>"Thomas Weber"</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>"thomas.weber.43@example.com"</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>"GDKKHGLEHELIINPJMCODNKGEGFOHJICDHPGODADPOMLEEEFEONNOBKAG"</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>The cost optimizer showed me exactly how much I saved.</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>4b971854a90c57f71bc8792cb774ad1912a74e3134f57ff1eb8f9e93d83fe800</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>"Viktor Novak"</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>"viktor.novak.44@example.com"</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>"GDCGGDPAOKCNLCKONEENPHLCHNHELMMMGFEKMBJBHOEPPKGAEGMPIIML"</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Highly secure and instant transfers.</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>dabb86e402025c492f816afe2654b8a556c299ab126aff5592a1c8f87497d07a</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>"Angela Cruz"</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>"angela.cruz.45@example.com"</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>"GDMBKLCIDOPOIHJIAFBAFIOCMCILEIKONNKLCCKLDDEPHDKIBEEEHLGA"</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Paisa makes cross-border transfer so easy!</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>f2ecba1db077a84e85b233faff34f34c359c55d2cf7be1775c8dda9e03d297d3</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>"Christian Santos"</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>"christian.santos.46@example.com"</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>"GDCLMPDPDPAGFBPMPKIJMNFGBBCFEEGJLNFBEKPNKPEJMPAJMFCHPGEJ"</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Great UX with fee bumps.</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>166e55713a481dec9f47d068a1b259a7d7221dc58da9e3bcc0ce5f6d1ab0ac93</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>"Elisa Reyes"</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>"elisa.reyes.47@example.com"</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>"GDFLELLGBPCLKKJECGPLBELJHGOFOOPNNIHHEIMIDNEIBAHBMAPGDIEG"</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Very cheap rates and fast transaction times.</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>0c3187b73c692e99dbb3b74f5f642bb9a714419c43397ecc9bf7897f8f542e64</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>"Gabriel Aquino"</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>"gabriel.aquino.48@example.com"</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>"GDLFIKMEKMNIIPOCEKMIBOFIIPPOGDOOIEFCOPAFOOABPJAJNIIIIMEE"</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>Incredibly user-friendly interface.</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>77e852154bb998a22d2d4cad5023c452028fc7fa772f1d3e24ae26a9b431d421</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>"Janice Perez"</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>"janice.perez.49@example.com"</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>"GDJFGPOCIOFDKPDMCGBHCHDNJLEGCPCKJNEIHGBNIABHCEHANKKFIFCJ"</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>Stellar Mainnet transfers are lightning fast.</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>0e2e2c119d9de95655e95a75a2852f9e318c3201915b2ffd916374b8ca3f5b84</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>"Lito Ramos"</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>"lito.ramos.50@example.com"</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>"GDLDPGLBIIMCMPNPJGKDELIPJIJCGJIHBABLFKJNBBIAALAOGMDHEBDC"</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>Happy with the conversion rates.</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>e258ae3587fa7e076cd29e83f502de71403bdcf75d06c81293f2d67bd013a044</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>"Maria Santos"</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>"maria.santos.51@example.com"</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>"GDDKHDNHEPEOJFJJEOGGBEPDHEOLKAKKKECKKAADINGLOKHEDPPBMBOK"</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>KYC onboarding was super smooth.</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>d4228ea59e46a38040b738e10672026f0abad2741fa6f3c8e220ee01d1d646eb</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>"Melchor Ortiz"</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>"melchor.ortiz.52@example.com"</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>"GDDBOEMPNJFBNHDBNKLKCLLJDDBDCGNIEMPMDGCMEADLCDBNHFGPDPLI"</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>"INR"</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>I love the rate alerts console.</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>634ee9f6f12086cd1efee1f727cd27553007ea3260f8c1874d4cf643461047f1</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>2026-08-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>"Ramon Santos"</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>"ramon.santos.53@example.com"</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>"GDCHKFOCNIGLKOMPKIFEJLKIMPIBDLBJABMLLBAFHEHIEJFGNFDNPBLG"</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>"EUR"</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>The cost optimizer showed me exactly how much I saved.</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>1c670a8a6346d4d30275f0082ea9e7e00d2e255d02f4e0d11c51cee78c180550</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>"Teresa Aquino"</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>"teresa.aquino.54@example.com"</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>"GDDBNNODMBGDCLMHHDNFDFCJMDJAAHMMNKEHDHFEFBBNOKKCJCDALOGF"</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>"PHP"</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>Highly secure and instant transfers.</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>1796e52b1478e2e9e8f644742d528d62d1da62ddc154f0d9d08b54aae6403011</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>